<commit_message>
Rebuild the artwork worklist in the shape its generator now writes
The four cards that came out of the archive landed while the Accepted column was being
removed, so the committed spreadsheet was still the old eight-column one. Regenerated:
29 cards, seven columns, and the fingerprint of the new content.

Both derived worklists carry the uncommitted Mbappe 97 to 96 that is in the working tree,
which moves his 2026 card from Monumental to Iconic. The next sync refreshes them either
way; they are generated files and the two agreeing with each other matters more here than
matching a rating that is about to change.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/missing-sticker-art.xlsx
+++ b/docs/missing-sticker-art.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Missing art'!$A$1:$H$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Missing art'!$A$1:$G$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -66,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -75,9 +75,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -451,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -460,8 +457,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,12 +491,7 @@
           <t>Tier</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>File to add</t>
         </is>
@@ -524,19 +515,14 @@
         <v>2026</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Monumental</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+          <t>Iconic</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>fra-2026-10.webp</t>
         </is>
@@ -567,12 +553,7 @@
           <t>Iconic</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>ned-1974-14.webp</t>
         </is>
@@ -603,12 +584,7 @@
           <t>Iconic</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>nor-2026-9.webp</t>
         </is>
@@ -639,12 +615,7 @@
           <t>Iconic</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>arg-2026-10.webp</t>
         </is>
@@ -675,12 +646,7 @@
           <t>Iconic</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>ger-1970-13.webp</t>
         </is>
@@ -711,12 +677,7 @@
           <t>Iconic</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>esp-2026-16.webp</t>
         </is>
@@ -747,12 +708,7 @@
           <t>Iconic</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>esp-2026-19.webp</t>
         </is>
@@ -783,12 +739,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>bra-1970-8.webp</t>
         </is>
@@ -819,12 +770,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>ger-1970-4.webp</t>
         </is>
@@ -855,12 +801,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>fra-1982-12.webp</t>
         </is>
@@ -891,12 +832,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>bra-2026-7.webp</t>
         </is>
@@ -927,12 +863,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>eng-2026-10.webp</t>
         </is>
@@ -963,12 +894,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>fra-1982-10.webp</t>
         </is>
@@ -999,12 +925,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>bra-1970-11.webp</t>
         </is>
@@ -1035,12 +956,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>eng-1970-6.webp</t>
         </is>
@@ -1071,12 +987,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>ned-1974-13.webp</t>
         </is>
@@ -1107,12 +1018,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>pol-1974-12.webp</t>
         </is>
@@ -1143,12 +1049,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>ned-1978-12.webp</t>
         </is>
@@ -1179,12 +1080,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>ger-1982-11.webp</t>
         </is>
@@ -1215,12 +1111,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>pol-1982-20.webp</t>
         </is>
@@ -1251,12 +1142,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>bra-1982-10.webp</t>
         </is>
@@ -1287,12 +1173,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>fra-1986-10.webp</t>
         </is>
@@ -1323,12 +1204,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>esp-1986-9.webp</t>
         </is>
@@ -1359,12 +1235,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>eng-1986-10.webp</t>
         </is>
@@ -1395,12 +1266,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>den-1986-10.webp</t>
         </is>
@@ -1431,12 +1297,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>urs-1986-19.webp</t>
         </is>
@@ -1467,12 +1328,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>mar-2026-2.webp</t>
         </is>
@@ -1503,12 +1359,7 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>bel-2026-1.webp</t>
         </is>
@@ -1539,19 +1390,14 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>fra-2026-7.webp</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H30"/>
+  <autoFilter ref="A1:G30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1574,14 +1420,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Sticker art still to draw</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Card set last changed</t>
         </is>
@@ -1593,31 +1439,31 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>with the dataset at commit</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7756263</t>
+          <t>0121695</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Fingerprint</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>d1a704cc5f51f412</t>
+          <t>80a59723c9bb44b5</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Collectibles in the dataset</t>
         </is>
@@ -1627,7 +1473,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>With artwork</t>
         </is>
@@ -1638,7 +1484,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Missing (rows on the list)</t>
         </is>
@@ -1648,19 +1494,8 @@
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Of those, accepted as silhouettes</t>
-        </is>
-      </c>
-      <c r="B9">
-        <f>COUNTIF('Missing art'!$G$2:$G$30,"yes")</f>
-        <v/>
-      </c>
-    </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Missing by tier</t>
         </is>
@@ -1711,14 +1546,14 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Generated by `npm run ratings:sync`. Do not edit by hand: the next rating change rewrites this file, and every figure above is derived from the dataset at the commit named in B4.</t>
         </is>
@@ -1727,25 +1562,25 @@
     <row r="19"/>
     <row r="20"/>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>To draw a card: save the full-size PNG as art/stickers-src/&lt;id&gt;.png, where &lt;id&gt; is the file name in the last column minus .webp, then run `npm run ratings:sync`. It builds the small WebP the site serves and takes the card off the waiting list.</t>
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>To draw a card: save the full-size PNG as art/stickers-src/&lt;id&gt;.png, where &lt;id&gt; is the file name in the last column minus .webp, then run `npm run ratings:sync`. It builds the small WebP the site serves and takes the card off the list.</t>
         </is>
       </c>
     </row>
     <row r="23"/>
     <row r="24"/>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>A row saying NO in Accepted is failing the build right now: either draw it or accept it as a silhouette with `npm run ratings:sync -- --accept-all`.</t>
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Nothing here is broken or failing. A card with no artwork shows a silhouette at the same size in the album, so this is a worklist rather than a fault list. The command above names the cards that appeared since the last time it ran, which is how a rating change that creates a new collectible gets noticed.</t>
         </is>
       </c>
     </row>
     <row r="27"/>
     <row r="28"/>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>A card is one player at one tournament, so the same man needs a card for each. On this list: Michel Platini (1982 and 1986).</t>
         </is>

</xml_diff>